<commit_message>
Checking bugs + Updating Login Page and Adjusting Notificatioand SMS
</commit_message>
<xml_diff>
--- a/assets/Annex 5-TES New Form 3.xlsx
+++ b/assets/Annex 5-TES New Form 3.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\judej\ScholarDoc\assets\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{2405C2C4-F75E-432F-A3E5-F21BA28E38A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{DD087ABE-D4DE-4737-90FF-03028B440F35}"/>
@@ -15,9 +10,6 @@
   <sheets>
     <sheet name="Annex 5-TES New Form 3" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -466,20 +458,28 @@
   <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -509,30 +509,30 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -551,30 +551,73 @@
 </styleSheet>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Annex 5-TES New Form 1"/>
-      <sheetName val="Annex 5-TES New Form 2"/>
-      <sheetName val="TES Amount"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="10">
-          <cell r="B10" t="str">
-            <v>TES Batch (Insert Number) - semester and Academic Year</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>363220</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>165735</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="714375" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="image1.png" title="Image"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4978400" y="737235"/>
+          <a:ext cx="714375" cy="742950"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>693420</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>165735</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="723900" cy="742950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="image2.png" title="Image"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9589770" y="737235"/>
+          <a:ext cx="723900" cy="742950"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -782,14 +825,22 @@
   <dimension ref="A1:AA998"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="10.44140625" customWidth="1"/>
-    <col min="5" max="5" width="21" customWidth="1"/>
-    <col min="6" max="6" width="31.88671875" customWidth="1"/>
-    <col min="10" max="10" width="28.44140625" customWidth="1"/>
-    <col min="12" max="12" width="22.44140625" customWidth="1"/>
+    <col min="1" max="1" width="3" customWidth="1"/>
+    <col min="2" max="2" width="11" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="32" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="28.5" customWidth="1"/>
+    <col min="11" max="11" width="10" customWidth="1"/>
+    <col min="12" max="12" width="22.5" customWidth="1"/>
+    <col min="13" max="13" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" thickBot="1">
+    <row r="1" spans="1:27" ht="25.2" customHeight="1" thickBot="1">
       <c r="A1" s="2"/>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
@@ -818,7 +869,7 @@
       <c r="Z1" s="1"/>
       <c r="AA1" s="1"/>
     </row>
-    <row r="2" spans="1:27" ht="14.4">
+    <row r="2" spans="1:27" ht="20" customHeight="1">
       <c r="A2" s="13"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -849,7 +900,7 @@
       <c r="Z2" s="1"/>
       <c r="AA2" s="1"/>
     </row>
-    <row r="3" spans="1:27" ht="14.4">
+    <row r="3" spans="1:27" ht="20" customHeight="1">
       <c r="A3" s="13"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -878,7 +929,7 @@
       <c r="Z3" s="1"/>
       <c r="AA3" s="1"/>
     </row>
-    <row r="4" spans="1:27" ht="14.4">
+    <row r="4" spans="1:27" ht="15" customHeight="1">
       <c r="A4" s="13"/>
       <c r="B4" s="39" t="s">
         <v>51</v>
@@ -909,7 +960,7 @@
       <c r="Z4" s="1"/>
       <c r="AA4" s="1"/>
     </row>
-    <row r="5" spans="1:27" ht="14.4">
+    <row r="5" spans="1:27" ht="15" customHeight="1">
       <c r="A5" s="13"/>
       <c r="B5" s="38" t="s">
         <v>50</v>
@@ -940,7 +991,7 @@
       <c r="Z5" s="1"/>
       <c r="AA5" s="1"/>
     </row>
-    <row r="6" spans="1:27" ht="14.4">
+    <row r="6" spans="1:27" ht="15" customHeight="1">
       <c r="A6" s="13"/>
       <c r="B6" s="37" t="s">
         <v>49</v>
@@ -971,7 +1022,7 @@
       <c r="Z6" s="1"/>
       <c r="AA6" s="1"/>
     </row>
-    <row r="7" spans="1:27" ht="14.4">
+    <row r="7" spans="1:27" ht="15.6" customHeight="1">
       <c r="A7" s="13"/>
       <c r="B7" s="2"/>
       <c r="C7" s="1"/>
@@ -1000,7 +1051,7 @@
       <c r="Z7" s="1"/>
       <c r="AA7" s="1"/>
     </row>
-    <row r="8" spans="1:27" ht="15" customHeight="1">
+    <row r="8" spans="1:27" ht="48" customHeight="1">
       <c r="A8" s="13"/>
       <c r="B8" s="36" t="s">
         <v>48</v>
@@ -1031,11 +1082,12 @@
       <c r="Z8" s="1"/>
       <c r="AA8" s="1"/>
     </row>
-    <row r="9" spans="1:27" ht="15.6">
+    <row r="9" spans="1:27" ht="18" customHeight="1">
       <c r="A9" s="13"/>
-      <c r="B9" s="35" t="str">
-        <f>'[1]Annex 5-TES New Form 2'!B10</f>
-        <v>TES Batch (Insert Number) - semester and Academic Year</v>
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>TES Batch (Insert Number) - semester and Academic Year</t>
+        </is>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -1063,7 +1115,7 @@
       <c r="Z9" s="1"/>
       <c r="AA9" s="1"/>
     </row>
-    <row r="10" spans="1:27" ht="14.4">
+    <row r="10" spans="1:27" ht="15.6" customHeight="1">
       <c r="A10" s="13"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -1092,7 +1144,7 @@
       <c r="Z10" s="1"/>
       <c r="AA10" s="1"/>
     </row>
-    <row r="11" spans="1:27" ht="16.2" thickBot="1">
+    <row r="11" spans="1:27" ht="16.2" customHeight="1" thickBot="1">
       <c r="A11" s="13"/>
       <c r="B11" s="21"/>
       <c r="C11" s="21"/>
@@ -1123,7 +1175,7 @@
       <c r="Z11" s="1"/>
       <c r="AA11" s="1"/>
     </row>
-    <row r="12" spans="1:27" ht="14.4">
+    <row r="12" spans="1:27" ht="15" customHeight="1">
       <c r="A12" s="13"/>
       <c r="B12" s="7" t="s">
         <v>46</v>
@@ -1841,7 +1893,7 @@
       <c r="Z33" s="15"/>
       <c r="AA33" s="15"/>
     </row>
-    <row r="34" spans="1:27" ht="29.4" thickBot="1">
+    <row r="34" spans="1:27" ht="15.75" customHeight="1" thickBot="1">
       <c r="A34" s="13"/>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -1853,9 +1905,7 @@
       <c r="I34" s="9"/>
       <c r="J34" s="9"/>
       <c r="K34" s="9"/>
-      <c r="L34" s="14" t="s">
-        <v>10</v>
-      </c>
+      <c r="L34" s="14"/>
       <c r="M34" s="9"/>
       <c r="N34" s="1"/>
       <c r="O34" s="1"/>
@@ -1872,7 +1922,7 @@
       <c r="Z34" s="1"/>
       <c r="AA34" s="1"/>
     </row>
-    <row r="35" spans="1:27" thickBot="1">
+    <row r="35" spans="1:27" ht="15.75" customHeight="1" thickBot="1">
       <c r="A35" s="13"/>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -1901,7 +1951,7 @@
       <c r="Z35" s="1"/>
       <c r="AA35" s="1"/>
     </row>
-    <row r="36" spans="1:27" thickBot="1">
+    <row r="36" spans="1:27" ht="15.75" customHeight="1" thickBot="1">
       <c r="A36" s="13"/>
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
@@ -1930,7 +1980,7 @@
       <c r="Z36" s="1"/>
       <c r="AA36" s="1"/>
     </row>
-    <row r="37" spans="1:27" thickBot="1">
+    <row r="37" spans="1:27" ht="15.75" customHeight="1" thickBot="1">
       <c r="A37" s="13"/>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
@@ -1959,7 +2009,7 @@
       <c r="Z37" s="1"/>
       <c r="AA37" s="1"/>
     </row>
-    <row r="38" spans="1:27" thickBot="1">
+    <row r="38" spans="1:27" ht="15.75" customHeight="1" thickBot="1">
       <c r="A38" s="13"/>
       <c r="B38" s="9"/>
       <c r="C38" s="9"/>
@@ -1988,7 +2038,7 @@
       <c r="Z38" s="1"/>
       <c r="AA38" s="1"/>
     </row>
-    <row r="39" spans="1:27" thickBot="1">
+    <row r="39" spans="1:27" ht="15.75" customHeight="1" thickBot="1">
       <c r="A39" s="13"/>
       <c r="B39" s="9"/>
       <c r="C39" s="9"/>
@@ -29879,6 +29929,7 @@
   <headerFooter>
     <oddFooter>&amp;C&amp;P of</oddFooter>
   </headerFooter>
+  <drawing r:id="rId3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>